<commit_message>
feat(siberman): per-member gender for relay teams (member_gender)
Добавлены колонки "Пол пловца/велосипедиста/бегуна" в Excel-шаблон и новое
поле participants.member_gender (миграция 004) — реальный пол участника
эстафеты, отдельно от gender='E' (маркер формата, используемый в рейтингах).
Для личников member_gender дублирует gender.
</commit_message>
<xml_diff>
--- a/docs/siberman/excel_template_raw.xlsx
+++ b/docs/siberman/excel_template_raw.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS2"/>
+  <dimension ref="A1:AV2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -450,7 +450,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="15.3" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
@@ -461,50 +461,53 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="14.4" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="14.4" customWidth="1" min="25" max="25"/>
+    <col width="14.4" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
-    <col width="12.6" customWidth="1" min="29" max="29"/>
-    <col width="23.4" customWidth="1" min="30" max="30"/>
+    <col width="14.4" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="12" customWidth="1" min="32" max="32"/>
-    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="12.6" customWidth="1" min="32" max="32"/>
+    <col width="23.4" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
-    <col width="13.5" customWidth="1" min="35" max="35"/>
-    <col width="13.5" customWidth="1" min="36" max="36"/>
-    <col width="13.5" customWidth="1" min="37" max="37"/>
-    <col width="14.4" customWidth="1" min="38" max="38"/>
-    <col width="14.4" customWidth="1" min="39" max="39"/>
-    <col width="14.4" customWidth="1" min="40" max="40"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="13.5" customWidth="1" min="38" max="38"/>
+    <col width="13.5" customWidth="1" min="39" max="39"/>
+    <col width="13.5" customWidth="1" min="40" max="40"/>
     <col width="14.4" customWidth="1" min="41" max="41"/>
     <col width="14.4" customWidth="1" min="42" max="42"/>
-    <col width="15.3" customWidth="1" min="43" max="43"/>
-    <col width="15.3" customWidth="1" min="44" max="44"/>
-    <col width="22.5" customWidth="1" min="45" max="45"/>
+    <col width="14.4" customWidth="1" min="43" max="43"/>
+    <col width="14.4" customWidth="1" min="44" max="44"/>
+    <col width="14.4" customWidth="1" min="45" max="45"/>
+    <col width="15.3" customWidth="1" min="46" max="46"/>
+    <col width="15.3" customWidth="1" min="47" max="47"/>
+    <col width="22.5" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Плавание</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Вело день 1</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Вело день 2</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Бег</t>
         </is>
@@ -548,190 +551,205 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>Пол пловца</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>Велосипедист</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Пол велосипедиста</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Бегун</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Пол бегуна</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Страна</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Город</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>1,3 км</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>2,6 км</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>3,9 км</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>5,2 км</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>6,5 км</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>7,8 км</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Финиш 10 км</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>3 км</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>10 км</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>72 км (разворот)</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>135 км</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>142 км</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>Финиш 145 км</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>Стартовая минута</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>51 км</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
+      <c r="AD2" s="2" t="inlineStr">
         <is>
           <t>82 км</t>
         </is>
       </c>
-      <c r="AB2" s="2" t="inlineStr">
+      <c r="AE2" s="2" t="inlineStr">
         <is>
           <t>119 км</t>
         </is>
       </c>
-      <c r="AC2" s="2" t="inlineStr">
+      <c r="AF2" s="2" t="inlineStr">
         <is>
           <t>160 км (СШГЭС)</t>
         </is>
       </c>
-      <c r="AD2" s="2" t="inlineStr">
+      <c r="AG2" s="2" t="inlineStr">
         <is>
           <t>190 км (Кольцо Саяногорск)</t>
         </is>
       </c>
-      <c r="AE2" s="2" t="inlineStr">
+      <c r="AH2" s="2" t="inlineStr">
         <is>
           <t>203 км</t>
         </is>
       </c>
-      <c r="AF2" s="2" t="inlineStr">
+      <c r="AI2" s="2" t="inlineStr">
         <is>
           <t>265 км</t>
         </is>
       </c>
-      <c r="AG2" s="2" t="inlineStr">
+      <c r="AJ2" s="2" t="inlineStr">
         <is>
           <t>Финиш 276 км</t>
         </is>
       </c>
-      <c r="AH2" s="2" t="inlineStr">
+      <c r="AK2" s="2" t="inlineStr">
         <is>
           <t>1 круг (7 км)</t>
         </is>
       </c>
-      <c r="AI2" s="2" t="inlineStr">
+      <c r="AL2" s="2" t="inlineStr">
         <is>
           <t>2 круга (14 км)</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr">
+      <c r="AM2" s="2" t="inlineStr">
         <is>
           <t>3 круга (21 км)</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="inlineStr">
+      <c r="AN2" s="2" t="inlineStr">
         <is>
           <t>4 круга (28 км)</t>
         </is>
       </c>
-      <c r="AL2" s="2" t="inlineStr">
+      <c r="AO2" s="2" t="inlineStr">
         <is>
           <t>5 кругов (35 км)</t>
         </is>
       </c>
-      <c r="AM2" s="2" t="inlineStr">
+      <c r="AP2" s="2" t="inlineStr">
         <is>
           <t>6 кругов (42 км)</t>
         </is>
       </c>
-      <c r="AN2" s="2" t="inlineStr">
+      <c r="AQ2" s="2" t="inlineStr">
         <is>
           <t>7 кругов (49 км)</t>
         </is>
       </c>
-      <c r="AO2" s="2" t="inlineStr">
+      <c r="AR2" s="2" t="inlineStr">
         <is>
           <t>8 кругов (56 км)</t>
         </is>
       </c>
-      <c r="AP2" s="2" t="inlineStr">
+      <c r="AS2" s="2" t="inlineStr">
         <is>
           <t>9 кругов (63 км)</t>
         </is>
       </c>
-      <c r="AQ2" s="2" t="inlineStr">
+      <c r="AT2" s="2" t="inlineStr">
         <is>
           <t>10 кругов (70 км)</t>
         </is>
       </c>
-      <c r="AR2" s="2" t="inlineStr">
+      <c r="AU2" s="2" t="inlineStr">
         <is>
           <t>11 кругов (77 км)</t>
         </is>
       </c>
-      <c r="AS2" s="2" t="inlineStr">
+      <c r="AV2" s="2" t="inlineStr">
         <is>
           <t>12 кругов (84 км) - Финиш</t>
         </is>
@@ -739,10 +757,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="S1:X1"/>
-    <mergeCell ref="Y1:AG1"/>
-    <mergeCell ref="AH1:AS1"/>
-    <mergeCell ref="L1:R1"/>
+    <mergeCell ref="AB1:AJ1"/>
+    <mergeCell ref="O1:U1"/>
+    <mergeCell ref="AK1:AV1"/>
+    <mergeCell ref="V1:AA1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(siberman): astronomical bike checkpoint time + auto-computed vело-2 start
Судьи вносят на КТ вело (день 1 и день 2) астрономическое время вместо
elapsed. Парсер не меняется (агностичен к семантике времени) — конвертация
происходит в новой service.convert_bike_times_to_elapsed(), вызываемой
после парсинга. Старт гонки (день 1) задаётся в админке при загрузке.

Старт вело-2 больше не ручной ввод — считается автоматически по рангу
вело-1 (общий зачёт individual+relay): 08:00 + топ-5 интервал 3 мин,
далее 1 мин. Правило подтверждено на реальных данных 2025 года (round-trip
regression: bib144 ранг1→08:00:00 итог 22:23:47, побитовое совпадение).

bike_day2_handicap_s репурпознан под вычисленный старт без миграции БД
(колонка была write-only) — теперь читается и показывается в админке и на
публичной странице результатов.
</commit_message>
<xml_diff>
--- a/docs/siberman/excel_template_raw.xlsx
+++ b/docs/siberman/excel_template_raw.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV2"/>
+  <dimension ref="A1:AU2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -468,27 +468,26 @@
     <col width="12" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="14.4" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="12.6" customWidth="1" min="32" max="32"/>
-    <col width="23.4" customWidth="1" min="33" max="33"/>
+    <col width="12.6" customWidth="1" min="31" max="31"/>
+    <col width="23.4" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
     <col width="12" customWidth="1" min="35" max="35"/>
     <col width="12" customWidth="1" min="36" max="36"/>
-    <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="13.5" customWidth="1" min="37" max="37"/>
     <col width="13.5" customWidth="1" min="38" max="38"/>
     <col width="13.5" customWidth="1" min="39" max="39"/>
-    <col width="13.5" customWidth="1" min="40" max="40"/>
+    <col width="14.4" customWidth="1" min="40" max="40"/>
     <col width="14.4" customWidth="1" min="41" max="41"/>
     <col width="14.4" customWidth="1" min="42" max="42"/>
     <col width="14.4" customWidth="1" min="43" max="43"/>
     <col width="14.4" customWidth="1" min="44" max="44"/>
-    <col width="14.4" customWidth="1" min="45" max="45"/>
+    <col width="15.3" customWidth="1" min="45" max="45"/>
     <col width="15.3" customWidth="1" min="46" max="46"/>
-    <col width="15.3" customWidth="1" min="47" max="47"/>
-    <col width="22.5" customWidth="1" min="48" max="48"/>
+    <col width="22.5" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,7 +506,7 @@
           <t>Вело день 2</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Бег</t>
         </is>
@@ -651,105 +650,100 @@
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>Стартовая минута</t>
+          <t>51 км</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>51 км</t>
+          <t>82 км</t>
         </is>
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>82 км</t>
+          <t>119 км</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
         <is>
-          <t>119 км</t>
+          <t>160 км (СШГЭС)</t>
         </is>
       </c>
       <c r="AF2" s="2" t="inlineStr">
         <is>
-          <t>160 км (СШГЭС)</t>
+          <t>190 км (Кольцо Саяногорск)</t>
         </is>
       </c>
       <c r="AG2" s="2" t="inlineStr">
         <is>
-          <t>190 км (Кольцо Саяногорск)</t>
+          <t>203 км</t>
         </is>
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>203 км</t>
+          <t>265 км</t>
         </is>
       </c>
       <c r="AI2" s="2" t="inlineStr">
         <is>
-          <t>265 км</t>
+          <t>Финиш 276 км</t>
         </is>
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>Финиш 276 км</t>
+          <t>1 круг (7 км)</t>
         </is>
       </c>
       <c r="AK2" s="2" t="inlineStr">
         <is>
-          <t>1 круг (7 км)</t>
+          <t>2 круга (14 км)</t>
         </is>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>2 круга (14 км)</t>
+          <t>3 круга (21 км)</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>3 круга (21 км)</t>
+          <t>4 круга (28 км)</t>
         </is>
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>4 круга (28 км)</t>
+          <t>5 кругов (35 км)</t>
         </is>
       </c>
       <c r="AO2" s="2" t="inlineStr">
         <is>
-          <t>5 кругов (35 км)</t>
+          <t>6 кругов (42 км)</t>
         </is>
       </c>
       <c r="AP2" s="2" t="inlineStr">
         <is>
-          <t>6 кругов (42 км)</t>
+          <t>7 кругов (49 км)</t>
         </is>
       </c>
       <c r="AQ2" s="2" t="inlineStr">
         <is>
-          <t>7 кругов (49 км)</t>
+          <t>8 кругов (56 км)</t>
         </is>
       </c>
       <c r="AR2" s="2" t="inlineStr">
         <is>
-          <t>8 кругов (56 км)</t>
+          <t>9 кругов (63 км)</t>
         </is>
       </c>
       <c r="AS2" s="2" t="inlineStr">
         <is>
-          <t>9 кругов (63 км)</t>
+          <t>10 кругов (70 км)</t>
         </is>
       </c>
       <c r="AT2" s="2" t="inlineStr">
         <is>
-          <t>10 кругов (70 км)</t>
+          <t>11 кругов (77 км)</t>
         </is>
       </c>
       <c r="AU2" s="2" t="inlineStr">
-        <is>
-          <t>11 кругов (77 км)</t>
-        </is>
-      </c>
-      <c r="AV2" s="2" t="inlineStr">
         <is>
           <t>12 кругов (84 км) - Финиш</t>
         </is>
@@ -757,9 +751,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="AB1:AJ1"/>
     <mergeCell ref="O1:U1"/>
-    <mergeCell ref="AK1:AV1"/>
+    <mergeCell ref="AJ1:AU1"/>
+    <mergeCell ref="AB1:AI1"/>
     <mergeCell ref="V1:AA1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>